<commit_message>
a couple of fixes base on class
</commit_message>
<xml_diff>
--- a/0-course-info/canvas/canvas_schedule.xlsx
+++ b/0-course-info/canvas/canvas_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/czmann/Documents/teaching/stat3540/0-course-info/canvas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B91504-18BC-DB4D-AA41-A543C9BC4D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66748238-5FDD-0B45-902D-516815C902C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17880" xr2:uid="{BA0A3FFF-9577-8249-B793-6919848B638A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="75">
   <si>
     <t>Week</t>
   </si>
@@ -264,6 +264,21 @@
   </si>
   <si>
     <t>Lab 3 data collection due 10/9</t>
+  </si>
+  <si>
+    <t>Activity 7.1</t>
+  </si>
+  <si>
+    <t>Lecture Video: Residuals aren't Normal
+Lecture Video: Non-Constant Variance
+Lecture Video: Non-Parametric Tests</t>
+  </si>
+  <si>
+    <t>Lecture Video: Intro to Causal Inference
+Lecture Video: Causal Inference with Randomized Experiments</t>
+  </si>
+  <si>
+    <t>Activity 8.1</t>
   </si>
 </sst>
 </file>
@@ -373,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -539,6 +554,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1317,9 +1335,9 @@
         <v>38</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="H21" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="H21" s="56" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1334,7 +1352,7 @@
       <c r="G22" s="55"/>
       <c r="H22" s="55"/>
     </row>
-    <row r="23" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="54">
         <v>8</v>
       </c>
@@ -1352,12 +1370,16 @@
       <c r="E23" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
+      <c r="F23" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>39</v>
+      </c>
       <c r="H23" s="18"/>
       <c r="I23" s="8"/>
     </row>
-    <row r="24" spans="1:9" ht="20.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="48" x14ac:dyDescent="0.2">
       <c r="A24" s="47"/>
       <c r="B24" s="4">
         <f>B23+1</f>
@@ -1372,6 +1394,12 @@
       </c>
       <c r="E24" s="6" t="s">
         <v>41</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G24" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="H24" s="26"/>
     </row>

</xml_diff>